<commit_message>
ajuistement de la page de profil
</commit_message>
<xml_diff>
--- a/storage/rapports/rapport_mensuel_2026-08-01_global.xlsx
+++ b/storage/rapports/rapport_mensuel_2026-08-01_global.xlsx
@@ -21,11 +21,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.0 &quot;h&quot;"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="[$-40C]#,##0"/>
+    <numFmt numFmtId="165" formatCode="[$-40C]#,##0.0 &quot;h&quot;"/>
+    <numFmt numFmtId="166" formatCode="[$-40C]0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,12 +36,21 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000F3D5C"/>
-      <sz val="15"/>
-    </font>
-    <font>
-      <color rgb="005B6B7A"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <color rgb="00D6E4EC"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="00D6E4EC"/>
+      <sz val="7.5"/>
     </font>
     <font>
       <i val="1"/>
@@ -49,25 +59,30 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="005B6B7A"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001C2733"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00D85A30"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="9.5"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001C2733"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="00D85A30"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00D85A30"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -82,12 +97,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="000F6E56"/>
+        <bgColor rgb="000F6E56"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F1FB"/>
+        <bgColor rgb="00E6F1FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAECE7"/>
+        <bgColor rgb="00FAECE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAEEDA"/>
+        <bgColor rgb="00FAEEDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F7F9FB"/>
         <bgColor rgb="00F7F9FB"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -102,6 +141,50 @@
       <right style="thin">
         <color rgb="00E1E5EA"/>
       </right>
+      <top style="thick">
+        <color rgb="000F3D5C"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E1E5EA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E1E5EA"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="00E1E5EA"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E1E5EA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E1E5EA"/>
+      </right>
+      <top style="thick">
+        <color rgb="00D85A30"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E1E5EA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E1E5EA"/>
+      </right>
+      <top style="thick">
+        <color rgb="00BA7517"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E1E5EA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E1E5EA"/>
+      </right>
       <top style="thin">
         <color rgb="00E1E5EA"/>
       </top>
@@ -113,33 +196,60 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="10" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -508,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -519,91 +629,114 @@
     <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Rapport mensuel de présence — Tous services</t>
         </is>
       </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>SRB Haute Matsiatra</t>
+        </is>
+      </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Du 01/08/2026 au 31/08/2026  •  Périmètre : Tous services</t>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Du 01/08/2026 au 31/08/2026</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Système de gestion biométrique des agents</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Généré le 03/08/2026 à 08:23 — document à usage interne</t>
-        </is>
-      </c>
+    <row r="3" ht="4" customHeight="1">
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Généré le 11/08/2026 à 09:01 — document à usage interne</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Agents concernés</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Taux de présence</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Retards</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Absences</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>Départs anticipés</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Heures travaillées</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="5" t="n">
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="n">
-        <v>0.0119</v>
-      </c>
-      <c r="C6" s="5" t="n">
+      <c r="B7" s="12" t="n">
+        <v>0.07140000000000001</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>0</v>
+      <c r="F7" s="15" t="n">
+        <v>0.19</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+  <mergeCells count="5">
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F1:G1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="1.2" right="1.2" top="1.4" bottom="1.2" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;9 Rapport mensuel de présence — Tous services</oddHeader>
-    <oddFooter>&amp;L&amp;8 Généré le 03/08/2026 à 08:23 — document à usage interne&amp;R&amp;8 Page &amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 Généré le 11/08/2026 à 09:01 — document à usage interne&amp;R&amp;8 Page &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -632,65 +765,65 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Agents</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>Taux de présence</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="16" t="inlineStr">
         <is>
           <t>Retards</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="16" t="inlineStr">
         <is>
           <t>Absences</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="16" t="inlineStr">
         <is>
           <t>Départs anticipés</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="16" t="inlineStr">
         <is>
           <t>Heures travaillées</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>Centre Informatique Régional</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n">
+      <c r="B2" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="C2" s="10" t="n">
-        <v>0.0119</v>
-      </c>
-      <c r="D2" s="9" t="n">
+      <c r="C2" s="19" t="n">
+        <v>0.07140000000000001</v>
+      </c>
+      <c r="D2" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="11" t="n">
-        <v>0</v>
+      <c r="G2" s="20" t="n">
+        <v>0.19</v>
       </c>
     </row>
   </sheetData>
@@ -700,7 +833,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;9 Rapport mensuel de présence — Tous services</oddHeader>
-    <oddFooter>&amp;L&amp;8 Généré le 03/08/2026 à 08:23 — document à usage interne&amp;R&amp;8 Page &amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 Généré le 11/08/2026 à 09:01 — document à usage interne&amp;R&amp;8 Page &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>